<commit_message>
Cập nhật test case.
</commit_message>
<xml_diff>
--- a/Extra/Test case.xlsx
+++ b/Extra/Test case.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lập Trình Mạng\PPTX\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8A10C3F-C2DD-4902-B08D-6A21449B1BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1029D160-8281-4B20-BBA7-DA815C0FA502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2088" yWindow="2100" windowWidth="20436" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Combined Test Cases" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -35,6 +35,62 @@
   </si>
   <si>
     <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>1. Open login page.
+2. Enter existing valid credentials.
+3. Click "Login" button.</t>
+  </si>
+  <si>
+    <t>Login successfully and redirect to the homepage.</t>
+  </si>
+  <si>
+    <t>Register</t>
+  </si>
+  <si>
+    <t>Register successfully, new account is created in the database.</t>
+  </si>
+  <si>
+    <t>System blocks registration and shows error: "Account already exists".</t>
+  </si>
+  <si>
+    <t>1. Open registration page.
+2. Enter a completely new username and password.
+3. Click "Register" button.</t>
+  </si>
+  <si>
+    <t>1. Open registration page.
+2. Enter an existing username.
+3. Click "Register" button.</t>
+  </si>
+  <si>
+    <t>Username: test1
+Password: 123</t>
+  </si>
+  <si>
+    <t>Username: test2
+Password: 123</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>System shows error: "Incorrect username or password".</t>
+  </si>
+  <si>
+    <t>System shows error: "Account already exists".</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
   </si>
 </sst>
 </file>
@@ -104,13 +160,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -119,9 +172,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -434,199 +493,317 @@
     <col min="3" max="3" width="60.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="42.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="53.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="28.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="3" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:8" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="5"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="5"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="5"/>
+      <c r="F1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="5"/>
+    </row>
+    <row r="2" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
+        <v>1</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H2" s="6"/>
+    </row>
+    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A3" s="4">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="6"/>
+    </row>
+    <row r="4" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="6"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+    </row>
+    <row r="8" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="1:8" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="5"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="6"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="6"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
-      <c r="B25" s="5"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sửa lỗi tính năng trả lời.
</commit_message>
<xml_diff>
--- a/Extra/Test case.xlsx
+++ b/Extra/Test case.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lập Trình Mạng\PPTX\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC65C8C-02FC-478D-90C1-4BEC42B7EC39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1AE93B-A7FF-4542-8E21-F226C9D59714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -599,11 +599,11 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="86.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="58.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="51.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="58" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="6.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Cập nhật test case, sửa tinh năng chuyển tiếp private chat.
</commit_message>
<xml_diff>
--- a/Extra/Test case.xlsx
+++ b/Extra/Test case.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lập Trình Mạng\PPTX\Extra\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lập Trình Mạng\Extra\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B381D503-EEC6-4A33-9C6D-A224631C2A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72BCB615-156F-4EDE-9213-7C68BD2EC7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1800" windowWidth="20436" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="75">
   <si>
     <t>Test Case ID</t>
-  </si>
-  <si>
-    <t>Function</t>
   </si>
   <si>
     <t>Test Steps</t>
@@ -81,12 +78,6 @@
 3. Click "Register" button.</t>
   </si>
   <si>
-    <t>System blocks registration and shows error: "Account already exists".</t>
-  </si>
-  <si>
-    <t>System shows error: "Account already exists".</t>
-  </si>
-  <si>
     <t>Group Chat</t>
   </si>
   <si>
@@ -180,29 +171,109 @@
     <t>Reply to Message</t>
   </si>
   <si>
+    <t>Reply text</t>
+  </si>
+  <si>
+    <t>The sent message is formatted as a reply.</t>
+  </si>
+  <si>
+    <t>Forward Message</t>
+  </si>
+  <si>
+    <t>Target user</t>
+  </si>
+  <si>
+    <t>The selected user receives the forwarded message successfully.</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Proof img_002</t>
+  </si>
+  <si>
+    <t>System shows error: "Tài khoản đã tồn tại".</t>
+  </si>
+  <si>
+    <t>System blocks registration and shows error: "Tài khoản đã tồn tại".</t>
+  </si>
+  <si>
     <t>1. Select text from an old message.
-2. Right-click and choose Reply.
+2. click and choose Reply.
 3. Type a reply and send.</t>
   </si>
   <si>
-    <t>Reply text</t>
-  </si>
-  <si>
-    <t>The sent message is formatted as a reply.</t>
-  </si>
-  <si>
-    <t>Forward Message</t>
-  </si>
-  <si>
-    <t>1. Select text from an old message
-2. Right-click and choose Forward
-3. Select a target user</t>
-  </si>
-  <si>
-    <t>Target user</t>
-  </si>
-  <si>
-    <t>The selected user receives the forwarded message successfully.</t>
+    <t>1. Select text from an old message.
+2. Click 'Forward' (Chuyển tiếp).
+3. Select a target user and click 'Gửi ngay'.</t>
+  </si>
+  <si>
+    <t>Send File (Private)</t>
+  </si>
+  <si>
+    <t>1. Open a private chat window.
+2. Click the 'Send File' button.
+3. Choose a valid file (e.g., .txt, .png, .docx) and send</t>
+  </si>
+  <si>
+    <t>A .txt or .png file</t>
+  </si>
+  <si>
+    <t>The file is uploaded and the receiver gets a notification/link to open the file.</t>
+  </si>
+  <si>
+    <t>Send Invalid File</t>
+  </si>
+  <si>
+    <t>1. Open a private chat window.
+2. Click the 'Send File' button.
+3. Choose an invalid file type (e.g., .exe, .bat).</t>
+  </si>
+  <si>
+    <t>An .exe file</t>
+  </si>
+  <si>
+    <t>System blocks the file transfer and shows an "Định dạng file không được hỗ trợ để đảm bảo an toàn!" error message.</t>
+  </si>
+  <si>
+    <t>Newline in Message</t>
+  </si>
+  <si>
+    <t>1. Type text into the chat input box.
+2. Press 'Shift + Enter'.
+3. Type more text and send.</t>
+  </si>
+  <si>
+    <t>Keystrokes: Shift+Enter</t>
+  </si>
+  <si>
+    <t>A new line is created in the input box, and the sent message contains multiple lines.</t>
+  </si>
+  <si>
+    <t>Empty Message</t>
+  </si>
+  <si>
+    <t>1. Leave the chat input box empty (or just spaces).
+2. Click the Send button or press Enter.</t>
+  </si>
+  <si>
+    <t>Empty string or spaces</t>
+  </si>
+  <si>
+    <t>The system ignores the action and prevents sending an empty message to the server.</t>
+  </si>
+  <si>
+    <t>Online Users List</t>
+  </si>
+  <si>
+    <t>1. Login with User A.
+2. Login with User B in another client.</t>
+  </si>
+  <si>
+    <t>Valid credentials for User B</t>
+  </si>
+  <si>
+    <t>User A's online list automatically updates to show User B is online without needing a refresh.</t>
   </si>
 </sst>
 </file>
@@ -258,13 +329,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -281,6 +355,583 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>22411</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>67234</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>4787</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1815353</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{49741554-DFE2-FF81-9B87-FBD87E9412CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18231970" y="246528"/>
+          <a:ext cx="2761435" cy="1748119"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>22412</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>11206</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>78441</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>1510787</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3F6F10AB-0B24-E5EC-2C0B-7EF68D648159}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18702618" y="2599765"/>
+          <a:ext cx="1624853" cy="1499581"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>33617</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>369794</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1580454</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{17DD81C8-C31E-9F7A-ABF7-590E7682AD3E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18680206" y="4179793"/>
+          <a:ext cx="4964206" cy="1546837"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>22412</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>56029</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>470646</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>1591954</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB964F67-FC65-F4A8-2A8C-1B6D5A1E77AE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18702618" y="5815853"/>
+          <a:ext cx="3227293" cy="1535925"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>201706</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>1499595</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{76A7A02A-FB47-97A6-5FF8-5537AB29DD89}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18680206" y="7933765"/>
+          <a:ext cx="2375647" cy="1499595"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>22411</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>67235</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>201706</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>1542351</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B81E1E58-BFCF-19C2-8004-F8DCFF62A7B1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18702617" y="9547411"/>
+          <a:ext cx="2353236" cy="1475116"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>201706</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>1497203</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE91EED7-D71A-A1EA-A3E4-889E89997A50}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18680206" y="11037794"/>
+          <a:ext cx="2375647" cy="1497203"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>587494</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>1748119</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D70C4CEE-5B24-4D5E-AC6D-FF5E7AE55277}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18680206" y="12561794"/>
+          <a:ext cx="2761435" cy="1748119"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>44824</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>33618</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>1732691</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1B9EAA2-E8B4-7C10-6BF8-AE5E4FC0EA2D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18725030" y="14377147"/>
+          <a:ext cx="2767853" cy="1732691"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>44823</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>284587</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>1714501</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{584EFB20-60C6-6F66-F269-3A95B6752465}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="18725029" y="16170089"/>
+          <a:ext cx="1808588" cy="1714500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>67236</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>67236</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>336177</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>1597262</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CEBEE3F-B486-6A7D-B507-5379A1B4C926}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19184471" y="18523324"/>
+          <a:ext cx="1837765" cy="1532267"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>60905</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>1882589</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{97B487D0-156C-34D5-E551-C3186260A0E2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19417553" y="20968448"/>
+          <a:ext cx="1029093" cy="1882588"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>331695</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>1160719</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F027D4BD-48DE-EAD4-0A75-0B316D72082C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="19417554" y="17893554"/>
+          <a:ext cx="2519082" cy="1160718"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -568,318 +1219,435 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="86.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="58.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="74.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="58" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="H1" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="146.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
-        <v>15</v>
-      </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="122.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="127.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" t="s">
-        <v>22</v>
-      </c>
       <c r="F5" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="127.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" t="s">
-        <v>28</v>
-      </c>
-      <c r="F7" t="s">
-        <v>29</v>
-      </c>
       <c r="G7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="121.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" t="s">
-        <v>33</v>
-      </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="123" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" t="s">
         <v>34</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" t="s">
-        <v>37</v>
-      </c>
       <c r="F9" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
         <v>38</v>
       </c>
-      <c r="C10" t="s">
+      <c r="F10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="142.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>39</v>
       </c>
-      <c r="D10" t="s">
+      <c r="C11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E10" t="s">
+      <c r="D11" t="s">
         <v>41</v>
       </c>
-      <c r="F10" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="E11" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11" t="s">
-        <v>45</v>
-      </c>
       <c r="F11" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="141" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F12" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="136.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="E13" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C14" s="2"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D14" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="127.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D15" t="s">
+        <v>61</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" t="s">
+        <v>26</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="151.19999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>